<commit_message>
commit mai 2026 #1
</commit_message>
<xml_diff>
--- a/pdf/TRISTAN DACQUIN - E5 Tableau de synthèse.xlsx
+++ b/pdf/TRISTAN DACQUIN - E5 Tableau de synthèse.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trifo\Documents\web\portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trifo\Documents\web\portfolio\pdf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D341DAB-7281-4715-BDCE-5830EB9912C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D04BF6E-5A28-4188-BE92-1FDF452C9675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,16 +50,10 @@
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
     <t>Option :</t>
   </si>
   <si>
     <t>▢ SLAM</t>
-  </si>
-  <si>
-    <t>Adresse URL du portfolio :</t>
   </si>
   <si>
     <t>Compétences mises en œuvre
@@ -217,6 +211,24 @@
       <t>(https://dacquin-tristan.fr)</t>
     </r>
   </si>
+  <si>
+    <t>Adresse URL du portfolio :     https://dacquin-tristan.fr</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">N° candidat : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2543708371</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -225,7 +237,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -298,6 +310,13 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -698,7 +717,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -763,6 +782,19 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -828,44 +860,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1198,124 +1192,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="29" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="30"/>
+      <c r="A3" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="35"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="A4" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="33"/>
       <c r="F4" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="13" t="s">
+    </row>
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="46" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="47"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="48"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="36" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="18" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
+      <c r="C6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="D6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="6" t="s">
+    </row>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="37"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="D7" s="19" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="19" t="s">
+      <c r="E7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="F7" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="G7" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="H7" s="20" t="s">
         <v>17</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="20" t="s">
-        <v>19</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1354,16 +1348,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="A8" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1400,875 +1394,875 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="50" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="44" t="s">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="15"/>
+      <c r="I9"/>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+      <c r="N9"/>
+      <c r="O9"/>
+      <c r="P9"/>
+      <c r="Q9"/>
+      <c r="R9"/>
+      <c r="S9"/>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
+      <c r="W9"/>
+      <c r="X9"/>
+      <c r="Y9"/>
+      <c r="Z9"/>
+      <c r="AA9"/>
+      <c r="AB9"/>
+      <c r="AC9"/>
+      <c r="AD9"/>
+      <c r="AE9"/>
+      <c r="AF9"/>
+      <c r="AG9"/>
+      <c r="AH9"/>
+      <c r="AI9"/>
+      <c r="AJ9"/>
+      <c r="AK9"/>
+      <c r="AL9"/>
+      <c r="AM9"/>
+      <c r="AN9"/>
+      <c r="AO9"/>
+      <c r="AP9"/>
+      <c r="AQ9"/>
+    </row>
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="15"/>
+      <c r="I10"/>
+      <c r="J10"/>
+      <c r="K10"/>
+      <c r="L10"/>
+      <c r="M10"/>
+      <c r="N10"/>
+      <c r="O10"/>
+      <c r="P10"/>
+      <c r="Q10"/>
+      <c r="R10"/>
+      <c r="S10"/>
+      <c r="T10"/>
+      <c r="U10"/>
+      <c r="V10"/>
+      <c r="W10"/>
+      <c r="X10"/>
+      <c r="Y10"/>
+      <c r="Z10"/>
+      <c r="AA10"/>
+      <c r="AB10"/>
+      <c r="AC10"/>
+      <c r="AD10"/>
+      <c r="AE10"/>
+      <c r="AF10"/>
+      <c r="AG10"/>
+      <c r="AH10"/>
+      <c r="AI10"/>
+      <c r="AJ10"/>
+      <c r="AK10"/>
+      <c r="AL10"/>
+      <c r="AM10"/>
+      <c r="AN10"/>
+      <c r="AO10"/>
+      <c r="AP10"/>
+      <c r="AQ10"/>
+    </row>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="45"/>
-      <c r="C9" s="46" t="s">
+      <c r="B11" s="8"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11"/>
+      <c r="J11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="N11"/>
+      <c r="O11"/>
+      <c r="P11"/>
+      <c r="Q11"/>
+      <c r="R11"/>
+      <c r="S11"/>
+      <c r="T11"/>
+      <c r="U11"/>
+      <c r="V11"/>
+      <c r="W11"/>
+      <c r="X11"/>
+      <c r="Y11"/>
+      <c r="Z11"/>
+      <c r="AA11"/>
+      <c r="AB11"/>
+      <c r="AC11"/>
+      <c r="AD11"/>
+      <c r="AE11"/>
+      <c r="AF11"/>
+      <c r="AG11"/>
+      <c r="AH11"/>
+      <c r="AI11"/>
+      <c r="AJ11"/>
+      <c r="AK11"/>
+      <c r="AL11"/>
+      <c r="AM11"/>
+      <c r="AN11"/>
+      <c r="AO11"/>
+      <c r="AP11"/>
+      <c r="AQ11"/>
+    </row>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="8"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="15"/>
+      <c r="I12"/>
+      <c r="J12"/>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12"/>
+      <c r="O12"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12"/>
+      <c r="U12"/>
+      <c r="V12"/>
+      <c r="W12"/>
+      <c r="X12"/>
+      <c r="Y12"/>
+      <c r="Z12"/>
+      <c r="AA12"/>
+      <c r="AB12"/>
+      <c r="AC12"/>
+      <c r="AD12"/>
+      <c r="AE12"/>
+      <c r="AF12"/>
+      <c r="AG12"/>
+      <c r="AH12"/>
+      <c r="AI12"/>
+      <c r="AJ12"/>
+      <c r="AK12"/>
+      <c r="AL12"/>
+      <c r="AM12"/>
+      <c r="AN12"/>
+      <c r="AO12"/>
+      <c r="AP12"/>
+      <c r="AQ12"/>
+    </row>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="15"/>
+      <c r="I13"/>
+      <c r="J13"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13"/>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13"/>
+      <c r="U13"/>
+      <c r="V13"/>
+      <c r="W13"/>
+      <c r="X13"/>
+      <c r="Y13"/>
+      <c r="Z13"/>
+      <c r="AA13"/>
+      <c r="AB13"/>
+      <c r="AC13"/>
+      <c r="AD13"/>
+      <c r="AE13"/>
+      <c r="AF13"/>
+      <c r="AG13"/>
+      <c r="AH13"/>
+      <c r="AI13"/>
+      <c r="AJ13"/>
+      <c r="AK13"/>
+      <c r="AL13"/>
+      <c r="AM13"/>
+      <c r="AN13"/>
+      <c r="AO13"/>
+      <c r="AP13"/>
+      <c r="AQ13"/>
+    </row>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="15"/>
+      <c r="I14"/>
+      <c r="J14"/>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14"/>
+      <c r="N14"/>
+      <c r="O14"/>
+      <c r="P14"/>
+      <c r="Q14"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14"/>
+      <c r="U14"/>
+      <c r="V14"/>
+      <c r="W14"/>
+      <c r="X14"/>
+      <c r="Y14"/>
+      <c r="Z14"/>
+      <c r="AA14"/>
+      <c r="AB14"/>
+      <c r="AC14"/>
+      <c r="AD14"/>
+      <c r="AE14"/>
+      <c r="AF14"/>
+      <c r="AG14"/>
+      <c r="AH14"/>
+      <c r="AI14"/>
+      <c r="AJ14"/>
+      <c r="AK14"/>
+      <c r="AL14"/>
+      <c r="AM14"/>
+      <c r="AN14"/>
+      <c r="AO14"/>
+      <c r="AP14"/>
+      <c r="AQ14"/>
+    </row>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="15"/>
+      <c r="I15"/>
+      <c r="J15"/>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15"/>
+      <c r="N15"/>
+      <c r="O15"/>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15"/>
+      <c r="V15"/>
+      <c r="W15"/>
+      <c r="X15"/>
+      <c r="Y15"/>
+      <c r="Z15"/>
+      <c r="AA15"/>
+      <c r="AB15"/>
+      <c r="AC15"/>
+      <c r="AD15"/>
+      <c r="AE15"/>
+      <c r="AF15"/>
+      <c r="AG15"/>
+      <c r="AH15"/>
+      <c r="AI15"/>
+      <c r="AJ15"/>
+      <c r="AK15"/>
+      <c r="AL15"/>
+      <c r="AM15"/>
+      <c r="AN15"/>
+      <c r="AO15"/>
+      <c r="AP15"/>
+      <c r="AQ15"/>
+    </row>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16"/>
+      <c r="J16"/>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16"/>
+      <c r="N16"/>
+      <c r="O16"/>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16"/>
+      <c r="V16"/>
+      <c r="W16"/>
+      <c r="X16"/>
+      <c r="Y16"/>
+      <c r="Z16"/>
+      <c r="AA16"/>
+      <c r="AB16"/>
+      <c r="AC16"/>
+      <c r="AD16"/>
+      <c r="AE16"/>
+      <c r="AF16"/>
+      <c r="AG16"/>
+      <c r="AH16"/>
+      <c r="AI16"/>
+      <c r="AJ16"/>
+      <c r="AK16"/>
+      <c r="AL16"/>
+      <c r="AM16"/>
+      <c r="AN16"/>
+      <c r="AO16"/>
+      <c r="AP16"/>
+      <c r="AQ16"/>
+    </row>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="I17"/>
+      <c r="J17"/>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
+      <c r="W17"/>
+      <c r="X17"/>
+      <c r="Y17"/>
+      <c r="Z17"/>
+      <c r="AA17"/>
+      <c r="AB17"/>
+      <c r="AC17"/>
+      <c r="AD17"/>
+      <c r="AE17"/>
+      <c r="AF17"/>
+      <c r="AG17"/>
+      <c r="AH17"/>
+      <c r="AI17"/>
+      <c r="AJ17"/>
+      <c r="AK17"/>
+      <c r="AL17"/>
+      <c r="AM17"/>
+      <c r="AN17"/>
+      <c r="AO17"/>
+      <c r="AP17"/>
+      <c r="AQ17"/>
+    </row>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="8"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="I18"/>
+      <c r="J18"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
+      <c r="W18"/>
+      <c r="X18"/>
+      <c r="Y18"/>
+      <c r="Z18"/>
+      <c r="AA18"/>
+      <c r="AB18"/>
+      <c r="AC18"/>
+      <c r="AD18"/>
+      <c r="AE18"/>
+      <c r="AF18"/>
+      <c r="AG18"/>
+      <c r="AH18"/>
+      <c r="AI18"/>
+      <c r="AJ18"/>
+      <c r="AK18"/>
+      <c r="AL18"/>
+      <c r="AM18"/>
+      <c r="AN18"/>
+      <c r="AO18"/>
+      <c r="AP18"/>
+      <c r="AQ18"/>
+    </row>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A19" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="43"/>
+      <c r="I19"/>
+      <c r="J19"/>
+      <c r="K19"/>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19"/>
+      <c r="O19"/>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
+      <c r="W19"/>
+      <c r="X19"/>
+      <c r="Y19"/>
+      <c r="Z19"/>
+      <c r="AA19"/>
+      <c r="AB19"/>
+      <c r="AC19"/>
+      <c r="AD19"/>
+      <c r="AE19"/>
+      <c r="AF19"/>
+      <c r="AG19"/>
+      <c r="AH19"/>
+      <c r="AI19"/>
+      <c r="AJ19"/>
+      <c r="AK19"/>
+      <c r="AL19"/>
+      <c r="AM19"/>
+      <c r="AN19"/>
+      <c r="AO19"/>
+      <c r="AP19"/>
+      <c r="AQ19"/>
+    </row>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="15"/>
+      <c r="I20"/>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+      <c r="W20"/>
+      <c r="X20"/>
+      <c r="Y20"/>
+      <c r="Z20"/>
+      <c r="AA20"/>
+      <c r="AB20"/>
+      <c r="AC20"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
+      <c r="AJ20"/>
+      <c r="AK20"/>
+      <c r="AL20"/>
+      <c r="AM20"/>
+      <c r="AN20"/>
+      <c r="AO20"/>
+      <c r="AP20"/>
+      <c r="AQ20"/>
+    </row>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="47"/>
-      <c r="E9" s="47"/>
-      <c r="F9" s="47"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="48"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="49"/>
-      <c r="N9" s="49"/>
-      <c r="O9" s="49"/>
-      <c r="P9" s="49"/>
-      <c r="Q9" s="49"/>
-      <c r="R9" s="49"/>
-      <c r="S9" s="49"/>
-      <c r="T9" s="49"/>
-      <c r="U9" s="49"/>
-      <c r="V9" s="49"/>
-      <c r="W9" s="49"/>
-      <c r="X9" s="49"/>
-      <c r="Y9" s="49"/>
-      <c r="Z9" s="49"/>
-      <c r="AA9" s="49"/>
-      <c r="AB9" s="49"/>
-      <c r="AC9" s="49"/>
-      <c r="AD9" s="49"/>
-      <c r="AE9" s="49"/>
-      <c r="AF9" s="49"/>
-      <c r="AG9" s="49"/>
-      <c r="AH9" s="49"/>
-      <c r="AI9" s="49"/>
-      <c r="AJ9" s="49"/>
-      <c r="AK9" s="49"/>
-      <c r="AL9" s="49"/>
-      <c r="AM9" s="49"/>
-      <c r="AN9" s="49"/>
-      <c r="AO9" s="49"/>
-      <c r="AP9" s="49"/>
-      <c r="AQ9" s="49"/>
-    </row>
-    <row r="10" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="48"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49"/>
-      <c r="L10" s="49"/>
-      <c r="M10" s="49"/>
-      <c r="N10" s="49"/>
-      <c r="O10" s="49"/>
-      <c r="P10" s="49"/>
-      <c r="Q10" s="49"/>
-      <c r="R10" s="49"/>
-      <c r="S10" s="49"/>
-      <c r="T10" s="49"/>
-      <c r="U10" s="49"/>
-      <c r="V10" s="49"/>
-      <c r="W10" s="49"/>
-      <c r="X10" s="49"/>
-      <c r="Y10" s="49"/>
-      <c r="Z10" s="49"/>
-      <c r="AA10" s="49"/>
-      <c r="AB10" s="49"/>
-      <c r="AC10" s="49"/>
-      <c r="AD10" s="49"/>
-      <c r="AE10" s="49"/>
-      <c r="AF10" s="49"/>
-      <c r="AG10" s="49"/>
-      <c r="AH10" s="49"/>
-      <c r="AI10" s="49"/>
-      <c r="AJ10" s="49"/>
-      <c r="AK10" s="49"/>
-      <c r="AL10" s="49"/>
-      <c r="AM10" s="49"/>
-      <c r="AN10" s="49"/>
-      <c r="AO10" s="49"/>
-      <c r="AP10" s="49"/>
-      <c r="AQ10" s="49"/>
-    </row>
-    <row r="11" spans="1:43" s="50" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="44" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="48"/>
-      <c r="I11" s="49"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="49"/>
-      <c r="L11" s="49"/>
-      <c r="M11" s="49"/>
-      <c r="N11" s="49"/>
-      <c r="O11" s="49"/>
-      <c r="P11" s="49"/>
-      <c r="Q11" s="49"/>
-      <c r="R11" s="49"/>
-      <c r="S11" s="49"/>
-      <c r="T11" s="49"/>
-      <c r="U11" s="49"/>
-      <c r="V11" s="49"/>
-      <c r="W11" s="49"/>
-      <c r="X11" s="49"/>
-      <c r="Y11" s="49"/>
-      <c r="Z11" s="49"/>
-      <c r="AA11" s="49"/>
-      <c r="AB11" s="49"/>
-      <c r="AC11" s="49"/>
-      <c r="AD11" s="49"/>
-      <c r="AE11" s="49"/>
-      <c r="AF11" s="49"/>
-      <c r="AG11" s="49"/>
-      <c r="AH11" s="49"/>
-      <c r="AI11" s="49"/>
-      <c r="AJ11" s="49"/>
-      <c r="AK11" s="49"/>
-      <c r="AL11" s="49"/>
-      <c r="AM11" s="49"/>
-      <c r="AN11" s="49"/>
-      <c r="AO11" s="49"/>
-      <c r="AP11" s="49"/>
-      <c r="AQ11" s="49"/>
-    </row>
-    <row r="12" spans="1:43" s="50" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="51" t="s">
+      <c r="B21" s="8"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="H21" s="15"/>
+      <c r="I21"/>
+      <c r="J21"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+      <c r="N21"/>
+      <c r="O21"/>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21"/>
+      <c r="V21"/>
+      <c r="W21"/>
+      <c r="X21"/>
+      <c r="Y21"/>
+      <c r="Z21"/>
+      <c r="AA21"/>
+      <c r="AB21"/>
+      <c r="AC21"/>
+      <c r="AD21"/>
+      <c r="AE21"/>
+      <c r="AF21"/>
+      <c r="AG21"/>
+      <c r="AH21"/>
+      <c r="AI21"/>
+      <c r="AJ21"/>
+      <c r="AK21"/>
+      <c r="AL21"/>
+      <c r="AM21"/>
+      <c r="AN21"/>
+      <c r="AO21"/>
+      <c r="AP21"/>
+      <c r="AQ21"/>
+    </row>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" s="15"/>
+      <c r="I22"/>
+      <c r="J22"/>
+      <c r="K22"/>
+      <c r="L22"/>
+      <c r="M22"/>
+      <c r="N22"/>
+      <c r="O22"/>
+      <c r="P22"/>
+      <c r="Q22"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22"/>
+      <c r="V22"/>
+      <c r="W22"/>
+      <c r="X22"/>
+      <c r="Y22"/>
+      <c r="Z22"/>
+      <c r="AA22"/>
+      <c r="AB22"/>
+      <c r="AC22"/>
+      <c r="AD22"/>
+      <c r="AE22"/>
+      <c r="AF22"/>
+      <c r="AG22"/>
+      <c r="AH22"/>
+      <c r="AI22"/>
+      <c r="AJ22"/>
+      <c r="AK22"/>
+      <c r="AL22"/>
+      <c r="AM22"/>
+      <c r="AN22"/>
+      <c r="AO22"/>
+      <c r="AP22"/>
+      <c r="AQ22"/>
+    </row>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="8"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="46" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="48"/>
-      <c r="I12" s="49"/>
-      <c r="J12" s="49"/>
-      <c r="K12" s="49"/>
-      <c r="L12" s="49"/>
-      <c r="M12" s="49"/>
-      <c r="N12" s="49"/>
-      <c r="O12" s="49"/>
-      <c r="P12" s="49"/>
-      <c r="Q12" s="49"/>
-      <c r="R12" s="49"/>
-      <c r="S12" s="49"/>
-      <c r="T12" s="49"/>
-      <c r="U12" s="49"/>
-      <c r="V12" s="49"/>
-      <c r="W12" s="49"/>
-      <c r="X12" s="49"/>
-      <c r="Y12" s="49"/>
-      <c r="Z12" s="49"/>
-      <c r="AA12" s="49"/>
-      <c r="AB12" s="49"/>
-      <c r="AC12" s="49"/>
-      <c r="AD12" s="49"/>
-      <c r="AE12" s="49"/>
-      <c r="AF12" s="49"/>
-      <c r="AG12" s="49"/>
-      <c r="AH12" s="49"/>
-      <c r="AI12" s="49"/>
-      <c r="AJ12" s="49"/>
-      <c r="AK12" s="49"/>
-      <c r="AL12" s="49"/>
-      <c r="AM12" s="49"/>
-      <c r="AN12" s="49"/>
-      <c r="AO12" s="49"/>
-      <c r="AP12" s="49"/>
-      <c r="AQ12" s="49"/>
-    </row>
-    <row r="13" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="51" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="46" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" s="47"/>
-      <c r="F13" s="47"/>
-      <c r="G13" s="46"/>
-      <c r="H13" s="48"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="49"/>
-      <c r="M13" s="49"/>
-      <c r="N13" s="49"/>
-      <c r="O13" s="49"/>
-      <c r="P13" s="49"/>
-      <c r="Q13" s="49"/>
-      <c r="R13" s="49"/>
-      <c r="S13" s="49"/>
-      <c r="T13" s="49"/>
-      <c r="U13" s="49"/>
-      <c r="V13" s="49"/>
-      <c r="W13" s="49"/>
-      <c r="X13" s="49"/>
-      <c r="Y13" s="49"/>
-      <c r="Z13" s="49"/>
-      <c r="AA13" s="49"/>
-      <c r="AB13" s="49"/>
-      <c r="AC13" s="49"/>
-      <c r="AD13" s="49"/>
-      <c r="AE13" s="49"/>
-      <c r="AF13" s="49"/>
-      <c r="AG13" s="49"/>
-      <c r="AH13" s="49"/>
-      <c r="AI13" s="49"/>
-      <c r="AJ13" s="49"/>
-      <c r="AK13" s="49"/>
-      <c r="AL13" s="49"/>
-      <c r="AM13" s="49"/>
-      <c r="AN13" s="49"/>
-      <c r="AO13" s="49"/>
-      <c r="AP13" s="49"/>
-      <c r="AQ13" s="49"/>
-    </row>
-    <row r="14" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="51"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="48"/>
-      <c r="I14" s="49"/>
-      <c r="J14" s="49"/>
-      <c r="K14" s="49"/>
-      <c r="L14" s="49"/>
-      <c r="M14" s="49"/>
-      <c r="N14" s="49"/>
-      <c r="O14" s="49"/>
-      <c r="P14" s="49"/>
-      <c r="Q14" s="49"/>
-      <c r="R14" s="49"/>
-      <c r="S14" s="49"/>
-      <c r="T14" s="49"/>
-      <c r="U14" s="49"/>
-      <c r="V14" s="49"/>
-      <c r="W14" s="49"/>
-      <c r="X14" s="49"/>
-      <c r="Y14" s="49"/>
-      <c r="Z14" s="49"/>
-      <c r="AA14" s="49"/>
-      <c r="AB14" s="49"/>
-      <c r="AC14" s="49"/>
-      <c r="AD14" s="49"/>
-      <c r="AE14" s="49"/>
-      <c r="AF14" s="49"/>
-      <c r="AG14" s="49"/>
-      <c r="AH14" s="49"/>
-      <c r="AI14" s="49"/>
-      <c r="AJ14" s="49"/>
-      <c r="AK14" s="49"/>
-      <c r="AL14" s="49"/>
-      <c r="AM14" s="49"/>
-      <c r="AN14" s="49"/>
-      <c r="AO14" s="49"/>
-      <c r="AP14" s="49"/>
-      <c r="AQ14" s="49"/>
-    </row>
-    <row r="15" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="51"/>
-      <c r="B15" s="45"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="47"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="48"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="49"/>
-      <c r="L15" s="49"/>
-      <c r="M15" s="49"/>
-      <c r="N15" s="49"/>
-      <c r="O15" s="49"/>
-      <c r="P15" s="49"/>
-      <c r="Q15" s="49"/>
-      <c r="R15" s="49"/>
-      <c r="S15" s="49"/>
-      <c r="T15" s="49"/>
-      <c r="U15" s="49"/>
-      <c r="V15" s="49"/>
-      <c r="W15" s="49"/>
-      <c r="X15" s="49"/>
-      <c r="Y15" s="49"/>
-      <c r="Z15" s="49"/>
-      <c r="AA15" s="49"/>
-      <c r="AB15" s="49"/>
-      <c r="AC15" s="49"/>
-      <c r="AD15" s="49"/>
-      <c r="AE15" s="49"/>
-      <c r="AF15" s="49"/>
-      <c r="AG15" s="49"/>
-      <c r="AH15" s="49"/>
-      <c r="AI15" s="49"/>
-      <c r="AJ15" s="49"/>
-      <c r="AK15" s="49"/>
-      <c r="AL15" s="49"/>
-      <c r="AM15" s="49"/>
-      <c r="AN15" s="49"/>
-      <c r="AO15" s="49"/>
-      <c r="AP15" s="49"/>
-      <c r="AQ15" s="49"/>
-    </row>
-    <row r="16" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="45"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="53" t="s">
-        <v>27</v>
-      </c>
-      <c r="I16" s="49"/>
-      <c r="J16" s="49"/>
-      <c r="K16" s="49"/>
-      <c r="L16" s="49"/>
-      <c r="M16" s="49"/>
-      <c r="N16" s="49"/>
-      <c r="O16" s="49"/>
-      <c r="P16" s="49"/>
-      <c r="Q16" s="49"/>
-      <c r="R16" s="49"/>
-      <c r="S16" s="49"/>
-      <c r="T16" s="49"/>
-      <c r="U16" s="49"/>
-      <c r="V16" s="49"/>
-      <c r="W16" s="49"/>
-      <c r="X16" s="49"/>
-      <c r="Y16" s="49"/>
-      <c r="Z16" s="49"/>
-      <c r="AA16" s="49"/>
-      <c r="AB16" s="49"/>
-      <c r="AC16" s="49"/>
-      <c r="AD16" s="49"/>
-      <c r="AE16" s="49"/>
-      <c r="AF16" s="49"/>
-      <c r="AG16" s="49"/>
-      <c r="AH16" s="49"/>
-      <c r="AI16" s="49"/>
-      <c r="AJ16" s="49"/>
-      <c r="AK16" s="49"/>
-      <c r="AL16" s="49"/>
-      <c r="AM16" s="49"/>
-      <c r="AN16" s="49"/>
-      <c r="AO16" s="49"/>
-      <c r="AP16" s="49"/>
-      <c r="AQ16" s="49"/>
-    </row>
-    <row r="17" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="47"/>
-      <c r="F17" s="47"/>
-      <c r="G17" s="47"/>
-      <c r="H17" s="53" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" s="49"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="49"/>
-      <c r="L17" s="49"/>
-      <c r="M17" s="49"/>
-      <c r="N17" s="49"/>
-      <c r="O17" s="49"/>
-      <c r="P17" s="49"/>
-      <c r="Q17" s="49"/>
-      <c r="R17" s="49"/>
-      <c r="S17" s="49"/>
-      <c r="T17" s="49"/>
-      <c r="U17" s="49"/>
-      <c r="V17" s="49"/>
-      <c r="W17" s="49"/>
-      <c r="X17" s="49"/>
-      <c r="Y17" s="49"/>
-      <c r="Z17" s="49"/>
-      <c r="AA17" s="49"/>
-      <c r="AB17" s="49"/>
-      <c r="AC17" s="49"/>
-      <c r="AD17" s="49"/>
-      <c r="AE17" s="49"/>
-      <c r="AF17" s="49"/>
-      <c r="AG17" s="49"/>
-      <c r="AH17" s="49"/>
-      <c r="AI17" s="49"/>
-      <c r="AJ17" s="49"/>
-      <c r="AK17" s="49"/>
-      <c r="AL17" s="49"/>
-      <c r="AM17" s="49"/>
-      <c r="AN17" s="49"/>
-      <c r="AO17" s="49"/>
-      <c r="AP17" s="49"/>
-      <c r="AQ17" s="49"/>
-    </row>
-    <row r="18" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="51" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="45"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="53" t="s">
-        <v>44</v>
-      </c>
-      <c r="F18" s="47"/>
-      <c r="G18" s="47"/>
-      <c r="I18" s="49"/>
-      <c r="J18" s="49"/>
-      <c r="K18" s="49"/>
-      <c r="L18" s="49"/>
-      <c r="M18" s="49"/>
-      <c r="N18" s="49"/>
-      <c r="O18" s="49"/>
-      <c r="P18" s="49"/>
-      <c r="Q18" s="49"/>
-      <c r="R18" s="49"/>
-      <c r="S18" s="49"/>
-      <c r="T18" s="49"/>
-      <c r="U18" s="49"/>
-      <c r="V18" s="49"/>
-      <c r="W18" s="49"/>
-      <c r="X18" s="49"/>
-      <c r="Y18" s="49"/>
-      <c r="Z18" s="49"/>
-      <c r="AA18" s="49"/>
-      <c r="AB18" s="49"/>
-      <c r="AC18" s="49"/>
-      <c r="AD18" s="49"/>
-      <c r="AE18" s="49"/>
-      <c r="AF18" s="49"/>
-      <c r="AG18" s="49"/>
-      <c r="AH18" s="49"/>
-      <c r="AI18" s="49"/>
-      <c r="AJ18" s="49"/>
-      <c r="AK18" s="49"/>
-      <c r="AL18" s="49"/>
-      <c r="AM18" s="49"/>
-      <c r="AN18" s="49"/>
-      <c r="AO18" s="49"/>
-      <c r="AP18" s="49"/>
-      <c r="AQ18" s="49"/>
-    </row>
-    <row r="19" spans="1:43" s="50" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="55"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="49"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="49"/>
-      <c r="N19" s="49"/>
-      <c r="O19" s="49"/>
-      <c r="P19" s="49"/>
-      <c r="Q19" s="49"/>
-      <c r="R19" s="49"/>
-      <c r="S19" s="49"/>
-      <c r="T19" s="49"/>
-      <c r="U19" s="49"/>
-      <c r="V19" s="49"/>
-      <c r="W19" s="49"/>
-      <c r="X19" s="49"/>
-      <c r="Y19" s="49"/>
-      <c r="Z19" s="49"/>
-      <c r="AA19" s="49"/>
-      <c r="AB19" s="49"/>
-      <c r="AC19" s="49"/>
-      <c r="AD19" s="49"/>
-      <c r="AE19" s="49"/>
-      <c r="AF19" s="49"/>
-      <c r="AG19" s="49"/>
-      <c r="AH19" s="49"/>
-      <c r="AI19" s="49"/>
-      <c r="AJ19" s="49"/>
-      <c r="AK19" s="49"/>
-      <c r="AL19" s="49"/>
-      <c r="AM19" s="49"/>
-      <c r="AN19" s="49"/>
-      <c r="AO19" s="49"/>
-      <c r="AP19" s="49"/>
-      <c r="AQ19" s="49"/>
-    </row>
-    <row r="20" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="45"/>
-      <c r="C20" s="53" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="49"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="49"/>
-      <c r="M20" s="49"/>
-      <c r="N20" s="49"/>
-      <c r="O20" s="49"/>
-      <c r="P20" s="49"/>
-      <c r="Q20" s="49"/>
-      <c r="R20" s="49"/>
-      <c r="S20" s="49"/>
-      <c r="T20" s="49"/>
-      <c r="U20" s="49"/>
-      <c r="V20" s="49"/>
-      <c r="W20" s="49"/>
-      <c r="X20" s="49"/>
-      <c r="Y20" s="49"/>
-      <c r="Z20" s="49"/>
-      <c r="AA20" s="49"/>
-      <c r="AB20" s="49"/>
-      <c r="AC20" s="49"/>
-      <c r="AD20" s="49"/>
-      <c r="AE20" s="49"/>
-      <c r="AF20" s="49"/>
-      <c r="AG20" s="49"/>
-      <c r="AH20" s="49"/>
-      <c r="AI20" s="49"/>
-      <c r="AJ20" s="49"/>
-      <c r="AK20" s="49"/>
-      <c r="AL20" s="49"/>
-      <c r="AM20" s="49"/>
-      <c r="AN20" s="49"/>
-      <c r="AO20" s="49"/>
-      <c r="AP20" s="49"/>
-      <c r="AQ20" s="49"/>
-    </row>
-    <row r="21" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="51" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="45"/>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="H21" s="48"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="49"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="49"/>
-      <c r="P21" s="49"/>
-      <c r="Q21" s="49"/>
-      <c r="R21" s="49"/>
-      <c r="S21" s="49"/>
-      <c r="T21" s="49"/>
-      <c r="U21" s="49"/>
-      <c r="V21" s="49"/>
-      <c r="W21" s="49"/>
-      <c r="X21" s="49"/>
-      <c r="Y21" s="49"/>
-      <c r="Z21" s="49"/>
-      <c r="AA21" s="49"/>
-      <c r="AB21" s="49"/>
-      <c r="AC21" s="49"/>
-      <c r="AD21" s="49"/>
-      <c r="AE21" s="49"/>
-      <c r="AF21" s="49"/>
-      <c r="AG21" s="49"/>
-      <c r="AH21" s="49"/>
-      <c r="AI21" s="49"/>
-      <c r="AJ21" s="49"/>
-      <c r="AK21" s="49"/>
-      <c r="AL21" s="49"/>
-      <c r="AM21" s="49"/>
-      <c r="AN21" s="49"/>
-      <c r="AO21" s="49"/>
-      <c r="AP21" s="49"/>
-      <c r="AQ21" s="49"/>
-    </row>
-    <row r="22" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="53" t="s">
-        <v>30</v>
-      </c>
-      <c r="H22" s="48"/>
-      <c r="I22" s="49"/>
-      <c r="J22" s="49"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="49"/>
-      <c r="M22" s="49"/>
-      <c r="N22" s="49"/>
-      <c r="O22" s="49"/>
-      <c r="P22" s="49"/>
-      <c r="Q22" s="49"/>
-      <c r="R22" s="49"/>
-      <c r="S22" s="49"/>
-      <c r="T22" s="49"/>
-      <c r="U22" s="49"/>
-      <c r="V22" s="49"/>
-      <c r="W22" s="49"/>
-      <c r="X22" s="49"/>
-      <c r="Y22" s="49"/>
-      <c r="Z22" s="49"/>
-      <c r="AA22" s="49"/>
-      <c r="AB22" s="49"/>
-      <c r="AC22" s="49"/>
-      <c r="AD22" s="49"/>
-      <c r="AE22" s="49"/>
-      <c r="AF22" s="49"/>
-      <c r="AG22" s="49"/>
-      <c r="AH22" s="49"/>
-      <c r="AI22" s="49"/>
-      <c r="AJ22" s="49"/>
-      <c r="AK22" s="49"/>
-      <c r="AL22" s="49"/>
-      <c r="AM22" s="49"/>
-      <c r="AN22" s="49"/>
-      <c r="AO22" s="49"/>
-      <c r="AP22" s="49"/>
-      <c r="AQ22" s="49"/>
-    </row>
-    <row r="23" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" s="45"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="53" t="s">
-        <v>43</v>
-      </c>
-      <c r="G23" s="47"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="49"/>
-      <c r="M23" s="49"/>
-      <c r="N23" s="49"/>
-      <c r="O23" s="49"/>
-      <c r="P23" s="49"/>
-      <c r="Q23" s="49"/>
-      <c r="R23" s="49"/>
-      <c r="S23" s="49"/>
-      <c r="T23" s="49"/>
-      <c r="U23" s="49"/>
-      <c r="V23" s="49"/>
-      <c r="W23" s="49"/>
-      <c r="X23" s="49"/>
-      <c r="Y23" s="49"/>
-      <c r="Z23" s="49"/>
-      <c r="AA23" s="49"/>
-      <c r="AB23" s="49"/>
-      <c r="AC23" s="49"/>
-      <c r="AD23" s="49"/>
-      <c r="AE23" s="49"/>
-      <c r="AF23" s="49"/>
-      <c r="AG23" s="49"/>
-      <c r="AH23" s="49"/>
-      <c r="AI23" s="49"/>
-      <c r="AJ23" s="49"/>
-      <c r="AK23" s="49"/>
-      <c r="AL23" s="49"/>
-      <c r="AM23" s="49"/>
-      <c r="AN23" s="49"/>
-      <c r="AO23" s="49"/>
-      <c r="AP23" s="49"/>
-      <c r="AQ23" s="49"/>
-    </row>
-    <row r="24" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="57"/>
-      <c r="B24" s="45"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="49"/>
-      <c r="M24" s="49"/>
-      <c r="N24" s="49"/>
-      <c r="O24" s="49"/>
-      <c r="P24" s="49"/>
-      <c r="Q24" s="49"/>
-      <c r="R24" s="49"/>
-      <c r="S24" s="49"/>
-      <c r="T24" s="49"/>
-      <c r="U24" s="49"/>
-      <c r="V24" s="49"/>
-      <c r="W24" s="49"/>
-      <c r="X24" s="49"/>
-      <c r="Y24" s="49"/>
-      <c r="Z24" s="49"/>
-      <c r="AA24" s="49"/>
-      <c r="AB24" s="49"/>
-      <c r="AC24" s="49"/>
-      <c r="AD24" s="49"/>
-      <c r="AE24" s="49"/>
-      <c r="AF24" s="49"/>
-      <c r="AG24" s="49"/>
-      <c r="AH24" s="49"/>
-      <c r="AI24" s="49"/>
-      <c r="AJ24" s="49"/>
-      <c r="AK24" s="49"/>
-      <c r="AL24" s="49"/>
-      <c r="AM24" s="49"/>
-      <c r="AN24" s="49"/>
-      <c r="AO24" s="49"/>
-      <c r="AP24" s="49"/>
-      <c r="AQ24" s="49"/>
-    </row>
-    <row r="25" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="57"/>
-      <c r="B25" s="45"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="47"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="49"/>
-      <c r="L25" s="49"/>
-      <c r="M25" s="49"/>
-      <c r="N25" s="49"/>
-      <c r="O25" s="49"/>
-      <c r="P25" s="49"/>
-      <c r="Q25" s="49"/>
-      <c r="R25" s="49"/>
-      <c r="S25" s="49"/>
-      <c r="T25" s="49"/>
-      <c r="U25" s="49"/>
-      <c r="V25" s="49"/>
-      <c r="W25" s="49"/>
-      <c r="X25" s="49"/>
-      <c r="Y25" s="49"/>
-      <c r="Z25" s="49"/>
-      <c r="AA25" s="49"/>
-      <c r="AB25" s="49"/>
-      <c r="AC25" s="49"/>
-      <c r="AD25" s="49"/>
-      <c r="AE25" s="49"/>
-      <c r="AF25" s="49"/>
-      <c r="AG25" s="49"/>
-      <c r="AH25" s="49"/>
-      <c r="AI25" s="49"/>
-      <c r="AJ25" s="49"/>
-      <c r="AK25" s="49"/>
-      <c r="AL25" s="49"/>
-      <c r="AM25" s="49"/>
-      <c r="AN25" s="49"/>
-      <c r="AO25" s="49"/>
-      <c r="AP25" s="49"/>
-      <c r="AQ25" s="49"/>
-    </row>
-    <row r="26" spans="1:43" s="50" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="57"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="49"/>
-      <c r="L26" s="49"/>
-      <c r="M26" s="49"/>
-      <c r="N26" s="49"/>
-      <c r="O26" s="49"/>
-      <c r="P26" s="49"/>
-      <c r="Q26" s="49"/>
-      <c r="R26" s="49"/>
-      <c r="S26" s="49"/>
-      <c r="T26" s="49"/>
-      <c r="U26" s="49"/>
-      <c r="V26" s="49"/>
-      <c r="W26" s="49"/>
-      <c r="X26" s="49"/>
-      <c r="Y26" s="49"/>
-      <c r="Z26" s="49"/>
-      <c r="AA26" s="49"/>
-      <c r="AB26" s="49"/>
-      <c r="AC26" s="49"/>
-      <c r="AD26" s="49"/>
-      <c r="AE26" s="49"/>
-      <c r="AF26" s="49"/>
-      <c r="AG26" s="49"/>
-      <c r="AH26" s="49"/>
-      <c r="AI26" s="49"/>
-      <c r="AJ26" s="49"/>
-      <c r="AK26" s="49"/>
-      <c r="AL26" s="49"/>
-      <c r="AM26" s="49"/>
-      <c r="AN26" s="49"/>
-      <c r="AO26" s="49"/>
-      <c r="AP26" s="49"/>
-      <c r="AQ26" s="49"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="15"/>
+      <c r="I23"/>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+      <c r="U23"/>
+      <c r="V23"/>
+      <c r="W23"/>
+      <c r="X23"/>
+      <c r="Y23"/>
+      <c r="Z23"/>
+      <c r="AA23"/>
+      <c r="AB23"/>
+      <c r="AC23"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23"/>
+      <c r="AH23"/>
+      <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
+    </row>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="15"/>
+      <c r="I24"/>
+      <c r="J24"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="Q24"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
+      <c r="W24"/>
+      <c r="X24"/>
+      <c r="Y24"/>
+      <c r="Z24"/>
+      <c r="AA24"/>
+      <c r="AB24"/>
+      <c r="AC24"/>
+      <c r="AD24"/>
+      <c r="AE24"/>
+      <c r="AF24"/>
+      <c r="AG24"/>
+      <c r="AH24"/>
+      <c r="AI24"/>
+      <c r="AJ24"/>
+      <c r="AK24"/>
+      <c r="AL24"/>
+      <c r="AM24"/>
+      <c r="AN24"/>
+      <c r="AO24"/>
+      <c r="AP24"/>
+      <c r="AQ24"/>
+    </row>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="15"/>
+      <c r="I25"/>
+      <c r="J25"/>
+      <c r="K25"/>
+      <c r="L25"/>
+      <c r="M25"/>
+      <c r="N25"/>
+      <c r="O25"/>
+      <c r="P25"/>
+      <c r="Q25"/>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+      <c r="U25"/>
+      <c r="V25"/>
+      <c r="W25"/>
+      <c r="X25"/>
+      <c r="Y25"/>
+      <c r="Z25"/>
+      <c r="AA25"/>
+      <c r="AB25"/>
+      <c r="AC25"/>
+      <c r="AD25"/>
+      <c r="AE25"/>
+      <c r="AF25"/>
+      <c r="AG25"/>
+      <c r="AH25"/>
+      <c r="AI25"/>
+      <c r="AJ25"/>
+      <c r="AK25"/>
+      <c r="AL25"/>
+      <c r="AM25"/>
+      <c r="AN25"/>
+      <c r="AO25"/>
+      <c r="AP25"/>
+      <c r="AQ25"/>
+    </row>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="9"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="15"/>
+      <c r="I26"/>
+      <c r="J26"/>
+      <c r="K26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+      <c r="N26"/>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26"/>
+      <c r="V26"/>
+      <c r="W26"/>
+      <c r="X26"/>
+      <c r="Y26"/>
+      <c r="Z26"/>
+      <c r="AA26"/>
+      <c r="AB26"/>
+      <c r="AC26"/>
+      <c r="AD26"/>
+      <c r="AE26"/>
+      <c r="AF26"/>
+      <c r="AG26"/>
+      <c r="AH26"/>
+      <c r="AI26"/>
+      <c r="AJ26"/>
+      <c r="AK26"/>
+      <c r="AL26"/>
+      <c r="AM26"/>
+      <c r="AN26"/>
+      <c r="AO26"/>
+      <c r="AP26"/>
+      <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="38"/>
+      <c r="A27" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="43"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2729,7 +2723,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait"/>
+  <pageSetup paperSize="9" scale="15" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
@@ -2986,9 +2980,15 @@
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37217530-9D4A-4C2E-B68D-E0AAC7F4CCAE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="23772b38-e52f-4d27-a92c-393309642c0d"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="ab57e019-d6c0-4014-a98d-66b5ffb74f49"/>
-    <ds:schemaRef ds:uri="23772b38-e52f-4d27-a92c-393309642c0d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>